<commit_message>
Completar procesamiento de UPRA-EVA
</commit_message>
<xml_diff>
--- a/data/config/1001_2_crosswalk_armonizado.xlsx
+++ b/data/config/1001_2_crosswalk_armonizado.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniandes-my.sharepoint.com/personal/jc_alfonso2004_uniandes_edu_co/Documents/PEG/PEG-mining-agriculture/data/config/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uniandes-my.sharepoint.com/personal/jc_alfonso2004_uniandes_edu_co/Documents/60740638-d4d4-46a0-82fc-572aa4f9fdb6/PEG/PEG-mining-agriculture/data/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1031" documentId="11_1D7141F7081B8D16392D4C2DEDED1FDF7879A7CD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0757255C-4400-4146-B950-E0467FE8F129}"/>
+  <xr:revisionPtr revIDLastSave="1045" documentId="11_1D7141F7081B8D16392D4C2DEDED1FDF7879A7CD" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5BF25226-9FB4-41E5-A647-EB87044EA9F2}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -54,8 +54,30 @@
 </comments>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3126" uniqueCount="436">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3128" uniqueCount="438">
   <si>
     <t>ciclo_original</t>
   </si>
@@ -1363,6 +1385,12 @@
   </si>
   <si>
     <t>|</t>
+  </si>
+  <si>
+    <t>Ciclos únicos</t>
+  </si>
+  <si>
+    <t>Grupos únicos</t>
   </si>
 </sst>
 </file>
@@ -5578,13 +5606,13 @@
         <v>366</v>
       </c>
       <c r="G95" s="6" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H95" s="6" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="I95" s="6" t="s">
-        <v>144</v>
+        <v>188</v>
       </c>
       <c r="K95" s="6" t="b">
         <v>1</v>
@@ -17789,18 +17817,19 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D435797-0EC0-43C3-AFE7-E830C34ABE90}">
-  <dimension ref="A2:B4"/>
+  <dimension ref="A2:E15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="23.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>375</v>
       </c>
@@ -17809,13 +17838,75 @@
         <v>60334863.758557297</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>379</v>
       </c>
       <c r="B4" s="3">
         <f>SUMIF(Sheet1!$E:$E,$A4,Sheet1!$D:$D)</f>
         <v>32491336.820000004</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>436</v>
+      </c>
+      <c r="B7" t="str" cm="1">
+        <f t="array" ref="B7:B9">_xlfn.UNIQUE(Sheet1!G2:G410)</f>
+        <v>Permanente</v>
+      </c>
+      <c r="D7" t="s">
+        <v>437</v>
+      </c>
+      <c r="E7" t="str" cm="1">
+        <f t="array" ref="E7:E15">_xlfn._xlws.SORT(_xlfn.UNIQUE(Sheet1!H2:H410),,-1)</f>
+        <v>Raíces y tubérculos</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B8" t="str">
+        <v>Transitorio</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Oleaginosas</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B9">
+        <v>0</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Leguminosas</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E10" t="str">
+        <v>Hortalizas</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E11" t="str">
+        <v>Frutales</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E12" t="str">
+        <v>Cultivos tropicales tradicionales</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E13" t="str">
+        <v>Cultivos para condimentos, bebidas medicinales y aromáticas</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E14" t="str">
+        <v>Cereales</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="E15">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>